<commit_message>
Drop Sources Shown? and Notes columns from evaluation report
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/evaluation_report.xlsx
+++ b/reports/evaluation_report.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -471,27 +471,17 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Sources Shown?</t>
+          <t>Confidence</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Confidence</t>
+          <t>Risk Flag</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Risk Flag</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
           <t>Pass / Fail</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Notes</t>
         </is>
       </c>
     </row>
@@ -521,25 +511,19 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Yes -- 6 catalog docs, confirmed correct across repeated runs.</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I2" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n"/>
+          <t>Pass</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -567,27 +551,17 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent. One repeat run mis-tagged Risk as 'Pricing' for this question; the other two runs agreed on 'None', taken as the reliable value.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -617,27 +591,17 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -667,27 +631,17 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -717,27 +671,17 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>Certification</t>
-        </is>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent. Consistent across all repeat runs.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -767,27 +711,17 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
           <t>Review</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent. Expected behavior assumed wireless is undocumented for any product; the app instead surfaces a customization-option caveat from the source docs. Worth a manual check of whether that customization claim is genuinely in the approved catalog text.</t>
         </is>
       </c>
     </row>
@@ -817,27 +751,17 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Certification</t>
-        </is>
-      </c>
-      <c r="I8" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent. Consistent across all repeat runs.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -867,27 +791,17 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Certification</t>
-        </is>
-      </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -917,27 +831,17 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Pricing</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Pricing</t>
-        </is>
-      </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent. No AURIGA price figure exists in the approved document set, so a full decline (rather than a caveated figure) is the correct, safer behavior. Consistent across all repeat runs.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -968,27 +872,17 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Pricing</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Pricing</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
           <t>Fail</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent. GAP: expected behavior assumes a 12-month warranty figure is approved content the app should state confidently. It instead declines. Consistent across all repeat runs -- either the 12-month figure is not actually present in the approved documents, or retrieval is missing it. Needs follow-up with whoever owns the approved-claims source docs.</t>
         </is>
       </c>
     </row>
@@ -1018,27 +912,17 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -1072,27 +956,17 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Accuracy</t>
-        </is>
-      </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -1122,27 +996,17 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I14" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -1187,27 +1051,17 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>High</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Certification</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>Certification</t>
-        </is>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent. Actual Answer is truncated at 2000 characters by the capture script (cuts off mid-word in the comparison table) -- not a re-run, the full answer was longer.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -1237,27 +1091,17 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Not reliably captured</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>None</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="inlineStr">
-        <is>
-          <t>Sources not independently verified for this row (see row 1) -- treat as unconfirmed, not absent.</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>

</xml_diff>